<commit_message>
Added 3 core commercial edge cases, chronological UTR sorting, and synchronized UI flags
</commit_message>
<xml_diff>
--- a/generated_data/bank_statement_union_bank.xlsx
+++ b/generated_data/bank_statement_union_bank.xlsx
@@ -450,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -496,22 +496,20 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>01-09-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>CMS/RAZORPAY/BATCH_SETL/CMS202609019237/CR</t>
+          <t>CMS/RAZORPAY/BATCH_SETL/CMS202605019455/CR</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n">
-        <v>3636.55</v>
-      </c>
+      <c r="F2" s="3" t="n"/>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>13,636.55 Cr</t>
+          <t>8,999.94 Cr</t>
         </is>
       </c>
     </row>
@@ -521,22 +519,22 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>02-09-2026</t>
+          <t>01-05-2026</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>CMS/RAZORPAY/BATCH_SETL/CMS202609023305/CR</t>
+          <t>UPIAB/539631629714/CR/TAIESWA/PPIW/6302476334.wal</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="3" t="n"/>
       <c r="F3" s="3" t="n">
-        <v>4496.71</v>
+        <v>368.88</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>18,133.26 Cr</t>
+          <t>9,368.82 Cr</t>
         </is>
       </c>
     </row>
@@ -546,22 +544,22 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>02-09-2026</t>
+          <t>02-05-2026</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>UPIAB/800823341214/CR/PITCHIKA/CNRB/ umanag9712@ax</t>
+          <t>CMS/RAZORPAY/BATCH_SETL/CMS202605023207/CR</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="3" t="n"/>
       <c r="F4" s="3" t="n">
-        <v>2169.46</v>
+        <v>438.89</v>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>20,302.72 Cr</t>
+          <t>9,807.71 Cr</t>
         </is>
       </c>
     </row>
@@ -571,22 +569,22 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>03-09-2026</t>
+          <t>02-05-2026</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>UPIAR/110099887766/DR/OLA CABS</t>
+          <t>INTEREST CREDIT / SBI SAVINGS &amp; CURRENT BAL</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="3" t="n">
-        <v>268.94</v>
-      </c>
-      <c r="F5" s="3" t="n"/>
+      <c r="E5" s="3" t="n"/>
+      <c r="F5" s="3" t="n">
+        <v>801.3099999999999</v>
+      </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>20,033.78 Cr</t>
+          <t>10,609.02 Cr</t>
         </is>
       </c>
     </row>
@@ -596,22 +594,22 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>04-09-2026</t>
+          <t>03-05-2026</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>CMS/RAZORPAY/BATCH_SETL/CMS202609042093/CR</t>
+          <t>CMS/RAZORPAY/BATCH_SETL/CMS202605036812/CR</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="3" t="n"/>
       <c r="F6" s="3" t="n">
-        <v>2247.28</v>
+        <v>4248.47</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>22,281.06 Cr</t>
+          <t>14,857.49 Cr</t>
         </is>
       </c>
     </row>
@@ -621,22 +619,22 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>05-09-2026</t>
+          <t>05-05-2026</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>CMS/RAZORPAY/BATCH_SETL/CMS202609053685/CR</t>
+          <t>CMS/RAZORPAY/BATCH_SETL/CMS202605052379/CR</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="3" t="n"/>
       <c r="F7" s="3" t="n">
-        <v>2317.1</v>
+        <v>3691.9</v>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>24,598.16 Cr</t>
+          <t>18,549.39 Cr</t>
         </is>
       </c>
     </row>
@@ -646,22 +644,22 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>06-09-2026</t>
+          <t>06-05-2026</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>CMS/RAZORPAY/BATCH_SETL/CMS202609062389/CR</t>
+          <t>CMS/RAZORPAY/BATCH_SETL/CMS202605067265/CR</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="3" t="n"/>
       <c r="F8" s="3" t="n">
-        <v>2439</v>
+        <v>1141.07</v>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>27,037.16 Cr</t>
+          <t>19,690.46 Cr</t>
         </is>
       </c>
     </row>
@@ -671,22 +669,22 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>06-09-2026</t>
+          <t>07-05-2026</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>UPIAR/665544332211/DR/AMAZON INDIA</t>
+          <t>CMS/RAZORPAY/BATCH_SETL/CMS202605076100/CR</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="3" t="n">
-        <v>1448.55</v>
-      </c>
-      <c r="F9" s="3" t="n"/>
+      <c r="E9" s="3" t="n"/>
+      <c r="F9" s="3" t="n">
+        <v>1580.98</v>
+      </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>25,588.61 Cr</t>
+          <t>21,271.44 Cr</t>
         </is>
       </c>
     </row>
@@ -696,22 +694,22 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>07-09-2026</t>
+          <t>08-05-2026</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>CMS/RAZORPAY/BATCH_SETL/CMS202609076328/CR</t>
+          <t>CMS/RAZORPAY/BATCH_SETL/CMS202605081706/CR</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="3" t="n"/>
       <c r="F10" s="3" t="n">
-        <v>802.84</v>
+        <v>1309.3</v>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>26,391.45 Cr</t>
+          <t>22,580.74 Cr</t>
         </is>
       </c>
     </row>
@@ -721,22 +719,22 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>07-09-2026</t>
+          <t>08-05-2026</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>UPIAB/322671730620/CR/PITCHIKA/SBIN/ 8919861154@ax</t>
+          <t>UPIAB/020074062699/CR/THIRUVEE/UBIN/9391652831-2@a</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="3" t="n"/>
       <c r="F11" s="3" t="n">
-        <v>1930.56</v>
+        <v>124.53</v>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>28,322.01 Cr</t>
+          <t>22,705.27 Cr</t>
         </is>
       </c>
     </row>
@@ -746,22 +744,22 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>08-09-2026</t>
+          <t>09-05-2026</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>CMS/RAZORPAY/BATCH_SETL/CMS202609081244/CR</t>
+          <t>CMS/RAZORPAY/BATCH_SETL/CMS202605095035/CR</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="3" t="n"/>
       <c r="F12" s="3" t="n">
-        <v>2445.15</v>
+        <v>5937.13</v>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>30,767.16 Cr</t>
+          <t>28,642.40 Cr</t>
         </is>
       </c>
     </row>
@@ -771,22 +769,22 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>09-09-2026</t>
+          <t>11-05-2026</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>CMS/RAZORPAY/BATCH_SETL/CMS202609098010/CR</t>
+          <t>UPIAB/443322110099/CR/PROMO DISCOUNT CREDIT</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="3" t="n"/>
       <c r="F13" s="3" t="n">
-        <v>4123.44</v>
+        <v>78.73999999999999</v>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>34,890.60 Cr</t>
+          <t>28,721.14 Cr</t>
         </is>
       </c>
     </row>
@@ -796,22 +794,22 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>09-09-2026</t>
+          <t>12-05-2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>UPIAR/026544681447/DR/SHANTIP/YESB/ Q707874078@yb</t>
+          <t>CMS/RAZORPAY/BATCH_SETL/CMS202605126192/CR</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="3" t="n">
-        <v>364.28</v>
-      </c>
-      <c r="F14" s="3" t="n"/>
+      <c r="E14" s="3" t="n"/>
+      <c r="F14" s="3" t="n">
+        <v>7131.43</v>
+      </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>34,526.32 Cr</t>
+          <t>35,852.57 Cr</t>
         </is>
       </c>
     </row>
@@ -821,22 +819,22 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>09-09-2026</t>
+          <t>13-05-2026</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>BANK SMS ALERTS &amp; ANNUAL MAINT CHARGES</t>
+          <t>CMS/RAZORPAY/BATCH_SETL/CMS202605138736/CR</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="3" t="n">
-        <v>92.34999999999999</v>
-      </c>
-      <c r="F15" s="3" t="n"/>
+      <c r="E15" s="3" t="n"/>
+      <c r="F15" s="3" t="n">
+        <v>1771.58</v>
+      </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>34,433.97 Cr</t>
+          <t>37,624.15 Cr</t>
         </is>
       </c>
     </row>
@@ -846,22 +844,22 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>10-09-2026</t>
+          <t>13-05-2026</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>CMS/RAZORPAY/BATCH_SETL/CMS202609106021/CR</t>
+          <t>UPIAR/204208208508/DR/Zomato87/AIRP/Zomato8759546.</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="3" t="n"/>
-      <c r="F16" s="3" t="n">
-        <v>2792.79</v>
-      </c>
+      <c r="E16" s="3" t="n">
+        <v>179.74</v>
+      </c>
+      <c r="F16" s="3" t="n"/>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>37,226.76 Cr</t>
+          <t>37,444.41 Cr</t>
         </is>
       </c>
     </row>
@@ -871,22 +869,22 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>11-09-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>CMS/RAZORPAY/BATCH_SETL/CMS202609115230/CR</t>
+          <t>CMS/RAZORPAY/BATCH_SETL/CMS202605144211/CR</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="3" t="n"/>
       <c r="F17" s="3" t="n">
-        <v>922.8</v>
+        <v>2730.17</v>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>38,149.56 Cr</t>
+          <t>40,174.58 Cr</t>
         </is>
       </c>
     </row>
@@ -896,22 +894,22 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>12-09-2026</t>
+          <t>14-05-2026</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>CMS/RAZORPAY/BATCH_SETL/CMS202609126886/CR</t>
+          <t>UPIAR/701074556047/DR/73374590/PUNB/7337459005@pty</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="3" t="n"/>
-      <c r="F18" s="3" t="n">
-        <v>4121.38</v>
-      </c>
+      <c r="E18" s="3" t="n">
+        <v>101.34</v>
+      </c>
+      <c r="F18" s="3" t="n"/>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>42,270.94 Cr</t>
+          <t>40,073.24 Cr</t>
         </is>
       </c>
     </row>
@@ -921,22 +919,22 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>12-09-2026</t>
+          <t>15-05-2026</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>UPIAR/140515780706/DR/ZOMATO/HDFC/payzomato@hdfc</t>
+          <t>CMS/RAZORPAY/BATCH_SETL/CMS202605152367/CR</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="3" t="n">
-        <v>187.91</v>
-      </c>
-      <c r="F19" s="3" t="n"/>
+      <c r="E19" s="3" t="n"/>
+      <c r="F19" s="3" t="n">
+        <v>1575.76</v>
+      </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>42,083.03 Cr</t>
+          <t>41,649.00 Cr</t>
         </is>
       </c>
     </row>
@@ -946,22 +944,22 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>12-09-2026</t>
+          <t>15-05-2026</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>UPIAR/455944913251/DR/KEMSARAP/SBIN/ 8977604821@yb</t>
+          <t>SHADOWFAX / DUNZO LAST MILE LOGISTICS FLEET</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="3" t="n">
-        <v>212.16</v>
+        <v>11223.4</v>
       </c>
       <c r="F20" s="3" t="n"/>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>41,870.87 Cr</t>
+          <t>30,425.60 Cr</t>
         </is>
       </c>
     </row>
@@ -971,22 +969,22 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>13-09-2026</t>
+          <t>16-05-2026</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>CMS/RAZORPAY/BATCH_SETL/CMS202609132900/CR</t>
+          <t>CMS/RAZORPAY/BATCH_SETL/CMS202605164710/CR</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="3" t="n"/>
       <c r="F21" s="3" t="n">
-        <v>243.07</v>
+        <v>3990.25</v>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>42,113.94 Cr</t>
+          <t>34,415.85 Cr</t>
         </is>
       </c>
     </row>
@@ -996,22 +994,22 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>13-09-2026</t>
+          <t>16-05-2026</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>UPIAR/812938102938/DR/PETROL PUMP/HPCL/hpcl@icici</t>
+          <t>OFFICE PANTRY &amp; FRESH REFRESHMENTS</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="3" t="n">
-        <v>774.59</v>
+        <v>1584.14</v>
       </c>
       <c r="F22" s="3" t="n"/>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>41,339.35 Cr</t>
+          <t>32,831.71 Cr</t>
         </is>
       </c>
     </row>
@@ -1021,22 +1019,22 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>14-09-2026</t>
+          <t>17-05-2026</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>CMS/RAZORPAY/BATCH_SETL/CMS202609144939/CR</t>
+          <t>CMS/RAZORPAY/BATCH_SETL/CMS202605178273/CR</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="3" t="n"/>
       <c r="F23" s="3" t="n">
-        <v>1266.14</v>
+        <v>1273.33</v>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>42,605.49 Cr</t>
+          <t>34,105.04 Cr</t>
         </is>
       </c>
     </row>
@@ -1046,22 +1044,22 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>15-09-2026</t>
+          <t>18-05-2026</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>CMS/RAZORPAY/BATCH_SETL/CMS202609151789/CR</t>
+          <t>CMS/RAZORPAY/BATCH_SETL/CMS202605189899/CR</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="3" t="n"/>
       <c r="F24" s="3" t="n">
-        <v>3049.01</v>
+        <v>1226.16</v>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>45,654.50 Cr</t>
+          <t>35,331.20 Cr</t>
         </is>
       </c>
     </row>
@@ -1071,22 +1069,22 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>16-09-2026</t>
+          <t>18-05-2026</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>CMS/RAZORPAY/BATCH_SETL/CMS202609166719/CR</t>
+          <t>UPIAB/322671730620/CR/PITCHIKA/SBIN/ 8919861154@ax</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="3" t="n"/>
       <c r="F25" s="3" t="n">
-        <v>3539.06</v>
+        <v>4367.77</v>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>49,193.56 Cr</t>
+          <t>39,698.97 Cr</t>
         </is>
       </c>
     </row>
@@ -1096,22 +1094,22 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>17-09-2026</t>
+          <t>19-05-2026</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>CMS/RAZORPAY/BATCH_SETL/CMS202609176485/CR</t>
+          <t>CMS/RAZORPAY/BATCH_SETL/CMS202605197998/CR</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr"/>
       <c r="E26" s="3" t="n"/>
       <c r="F26" s="3" t="n">
-        <v>6801.41</v>
+        <v>3120.03</v>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>55,994.97 Cr</t>
+          <t>42,819.00 Cr</t>
         </is>
       </c>
     </row>
@@ -1121,22 +1119,22 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>18-09-2026</t>
+          <t>20-05-2026</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>CMS/RAZORPAY/BATCH_SETL/CMS202609187785/CR</t>
+          <t>UPIAB/789123891023/CR/CUSTOMER REFUND REVERSAL</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr"/>
       <c r="E27" s="3" t="n"/>
       <c r="F27" s="3" t="n">
-        <v>3597.5</v>
+        <v>401.15</v>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>59,592.47 Cr</t>
+          <t>43,220.15 Cr</t>
         </is>
       </c>
     </row>
@@ -1146,22 +1144,22 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>18-09-2026</t>
+          <t>21-05-2026</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>UPIAR/123854061954/DR/ZOMATO/HDFC/payzomato@hdfc</t>
+          <t>CMS/RAZORPAY/BATCH_SETL/CMS202605214877/CR</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="3" t="n">
-        <v>266.91</v>
-      </c>
-      <c r="F28" s="3" t="n"/>
+      <c r="E28" s="3" t="n"/>
+      <c r="F28" s="3" t="n">
+        <v>4677.05</v>
+      </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>59,325.56 Cr</t>
+          <t>47,897.20 Cr</t>
         </is>
       </c>
     </row>
@@ -1171,22 +1169,22 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>19-09-2026</t>
+          <t>21-05-2026</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>CMS/RAZORPAY/BATCH_SETL/CMS202609199425/CR</t>
+          <t>SERVICE CHARGE / MINIMUM BALANCE FEE</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr"/>
-      <c r="E29" s="3" t="n"/>
-      <c r="F29" s="3" t="n">
-        <v>2167.4</v>
-      </c>
+      <c r="E29" s="3" t="n">
+        <v>385.41</v>
+      </c>
+      <c r="F29" s="3" t="n"/>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>61,492.96 Cr</t>
+          <t>47,511.79 Cr</t>
         </is>
       </c>
     </row>
@@ -1196,22 +1194,22 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>20-09-2026</t>
+          <t>21-05-2026</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>CMS/RAZORPAY/BATCH_SETL/CMS202609207527/CR</t>
+          <t>UPIAR/554433221100/DR/FLIPKART ONLINE</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="3" t="n"/>
-      <c r="F30" s="3" t="n">
-        <v>3197.76</v>
-      </c>
+      <c r="E30" s="3" t="n">
+        <v>2547.07</v>
+      </c>
+      <c r="F30" s="3" t="n"/>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>64,690.72 Cr</t>
+          <t>44,964.72 Cr</t>
         </is>
       </c>
     </row>
@@ -1221,22 +1219,22 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>21-09-2026</t>
+          <t>22-05-2026</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>CMS/RAZORPAY/BATCH_SETL/CMS202609215081/CR</t>
+          <t>CMS/RAZORPAY/BATCH_SETL/CMS202605227895/CR</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr"/>
       <c r="E31" s="3" t="n"/>
       <c r="F31" s="3" t="n">
-        <v>1981.85</v>
+        <v>563.87</v>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>66,672.57 Cr</t>
+          <t>45,528.59 Cr</t>
         </is>
       </c>
     </row>
@@ -1246,22 +1244,22 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>21-09-2026</t>
+          <t>22-05-2026</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>UPIAR/998877665544/DR/PAYTM QR VENDOR</t>
+          <t>WAREHOUSE STAFF WAGES &amp; PACKING CREW</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr"/>
       <c r="E32" s="3" t="n">
-        <v>72.2</v>
+        <v>26007.63</v>
       </c>
       <c r="F32" s="3" t="n"/>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>66,600.37 Cr</t>
+          <t>19,520.96 Cr</t>
         </is>
       </c>
     </row>
@@ -1271,22 +1269,22 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>21-09-2026</t>
+          <t>23-05-2026</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>PACKAGING SUPPLIES / ECO CORRUGATED BOXES</t>
+          <t>CMS/RAZORPAY/BATCH_SETL/CMS202605233589/CR</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr"/>
-      <c r="E33" s="3" t="n">
-        <v>10136.89</v>
-      </c>
-      <c r="F33" s="3" t="n"/>
+      <c r="E33" s="3" t="n"/>
+      <c r="F33" s="3" t="n">
+        <v>1834.21</v>
+      </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>56,463.48 Cr</t>
+          <t>21,355.17 Cr</t>
         </is>
       </c>
     </row>
@@ -1296,22 +1294,22 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>22-09-2026</t>
+          <t>24-05-2026</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>CMS/RAZORPAY/BATCH_SETL/CMS202609221181/CR</t>
+          <t>CMS/RAZORPAY/BATCH_SETL/CMS202605246400/CR</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="3" t="n"/>
       <c r="F34" s="3" t="n">
-        <v>1412.75</v>
+        <v>2316.07</v>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>57,876.23 Cr</t>
+          <t>23,671.24 Cr</t>
         </is>
       </c>
     </row>
@@ -1321,22 +1319,22 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>23-09-2026</t>
+          <t>25-05-2026</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>CMS/RAZORPAY/BATCH_SETL/CMS202609233081/CR</t>
+          <t>CMS/RAZORPAY/BATCH_SETL/CMS202605254539/CR</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="3" t="n"/>
       <c r="F35" s="3" t="n">
-        <v>697.15</v>
+        <v>178.48</v>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>58,573.38 Cr</t>
+          <t>23,849.72 Cr</t>
         </is>
       </c>
     </row>
@@ -1346,22 +1344,22 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>23-09-2026</t>
+          <t>26-05-2026</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>EMPLOYEE FIELD COMMUTE &amp; TRAVEL REIMBURSEMENT</t>
+          <t>CMS/RAZORPAY/BATCH_SETL/CMS202605269626/CR</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr"/>
-      <c r="E36" s="3" t="n">
-        <v>3968.31</v>
-      </c>
-      <c r="F36" s="3" t="n"/>
+      <c r="E36" s="3" t="n"/>
+      <c r="F36" s="3" t="n">
+        <v>1008.82</v>
+      </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>54,605.07 Cr</t>
+          <t>24,858.54 Cr</t>
         </is>
       </c>
     </row>
@@ -1371,122 +1369,22 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>24-09-2026</t>
+          <t>27-05-2026</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>CMS/RAZORPAY/BATCH_SETL/CMS202609241811/CR</t>
+          <t>CMS/RAZORPAY/BATCH_SETL/CMS202605277050/CR</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr"/>
       <c r="E37" s="3" t="n"/>
       <c r="F37" s="3" t="n">
-        <v>2465.65</v>
+        <v>149.78</v>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>57,070.72 Cr</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="n">
-        <v>37</v>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>25-09-2026</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>CMS/RAZORPAY/BATCH_SETL/CMS202609257127/CR</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr"/>
-      <c r="E38" s="3" t="n"/>
-      <c r="F38" s="3" t="n">
-        <v>2524.19</v>
-      </c>
-      <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t>59,594.91 Cr</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="n">
-        <v>38</v>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>25-09-2026</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>COMMERCIAL WAREHOUSE RENT / KORAMANGALA HUB</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr"/>
-      <c r="E39" s="3" t="n">
-        <v>49251.75</v>
-      </c>
-      <c r="F39" s="3" t="n"/>
-      <c r="G39" s="2" t="inlineStr">
-        <is>
-          <t>10,343.16 Cr</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="n">
-        <v>39</v>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>26-09-2026</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>CMS/RAZORPAY/BATCH_SETL/CMS202609267231/CR</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr"/>
-      <c r="E40" s="3" t="n"/>
-      <c r="F40" s="3" t="n">
-        <v>1121.6</v>
-      </c>
-      <c r="G40" s="2" t="inlineStr">
-        <is>
-          <t>11,464.76 Cr</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>27-09-2026</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>CMS/RAZORPAY/BATCH_SETL/CMS202609272822/CR</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr"/>
-      <c r="E41" s="3" t="n"/>
-      <c r="F41" s="3" t="n">
-        <v>1548.19</v>
-      </c>
-      <c r="G41" s="2" t="inlineStr">
-        <is>
-          <t>13,012.95 Cr</t>
+          <t>25,008.32 Cr</t>
         </is>
       </c>
     </row>

</xml_diff>